<commit_message>
chore: update progress tracker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/spreadsheet/startpray-progress-tracker.xlsx
+++ b/output/spreadsheet/startpray-progress-tracker.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>1ab8502</t>
+          <t>9cb3b86</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-12 14:44:50</t>
+          <t>2026-09-14 01:03:53</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5411,14 +5411,58 @@
           <t>[AUTO] Commit recorded: design/phase0-foundation @ 1ab8502</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
           <t>Continue task updates and prepare push.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-12 14:44:55</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: design/phase0-foundation @ 6dd5e0b</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>git-hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-09-14 01:03:53</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>[AUTO] Commit recorded: design/phase0-foundation @ 9cb3b86</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Continue task updates and prepare push.</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
         <is>
           <t>git-hook</t>
         </is>
@@ -5555,7 +5599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8500,7 +8544,81 @@
           <t>https://github.com/dan40912/Start-Pray.git</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-12 14:44:55</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>design/phase0-foundation</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>6dd5e0b</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>chore: update progress tracker</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-14 01:03:53</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>commit</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>design/phase0-foundation</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>9cb3b86</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>fix(voice): stop the countdown from restarting the recorder every second</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://github.com/dan40912/Start-Pray.git</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>